<commit_message>
starting to work on mpox params
</commit_message>
<xml_diff>
--- a/par-calculator.xlsx
+++ b/par-calculator.xlsx
@@ -1,28 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10908"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10720"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andres/code/operation-outbreak/oo-parameters/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0572FD19-5BB0-8547-A84C-93A513043F20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{463E801F-6E1A-7442-82F4-6D544E8B96C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3960" yWindow="500" windowWidth="38400" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EPI Calculation Formulas" sheetId="1" r:id="rId1"/>
     <sheet name="HPAI" sheetId="21" r:id="rId2"/>
-    <sheet name="TB" sheetId="9" r:id="rId3"/>
-    <sheet name="COVID" sheetId="11" r:id="rId4"/>
-    <sheet name="Marburg" sheetId="13" r:id="rId5"/>
-    <sheet name="Measles" sheetId="14" r:id="rId6"/>
-    <sheet name="Norovirus" sheetId="15" r:id="rId7"/>
-    <sheet name="Influenza" sheetId="17" r:id="rId8"/>
-    <sheet name="Stap" sheetId="18" r:id="rId9"/>
-    <sheet name="Disease X" sheetId="20" r:id="rId10"/>
+    <sheet name="mpox" sheetId="22" r:id="rId3"/>
+    <sheet name="TB" sheetId="9" r:id="rId4"/>
+    <sheet name="COVID" sheetId="11" r:id="rId5"/>
+    <sheet name="Marburg" sheetId="13" r:id="rId6"/>
+    <sheet name="Measles" sheetId="14" r:id="rId7"/>
+    <sheet name="Norovirus" sheetId="15" r:id="rId8"/>
+    <sheet name="Influenza" sheetId="17" r:id="rId9"/>
+    <sheet name="Stap" sheetId="18" r:id="rId10"/>
+    <sheet name="Disease X" sheetId="20" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="109">
   <si>
     <t>Simulation-independent parameters</t>
   </si>
@@ -383,6 +384,12 @@
   <si>
     <t>{"Saturday night fever":65,"Cough":100,"Stomach pain":50,"diarrhea":40}</t>
   </si>
+  <si>
+    <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC10468816/</t>
+  </si>
+  <si>
+    <t>Simulation-independent parameters for mpox</t>
+  </si>
 </sst>
 </file>
 
@@ -496,7 +503,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -548,8 +555,6 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -30481,6 +30486,224 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4966E832-9944-D544-886B-D77EBEEF54A6}">
+  <dimension ref="A1:D30"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <cols>
+    <col min="1" max="1" width="57.5" customWidth="1"/>
+    <col min="2" max="2" width="33" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A1" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="B1" s="25"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A2" s="3"/>
+      <c r="B2" s="3"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A4" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A5" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="3">
+        <v>0.14000000000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A6" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6">
+        <v>7.0000000000000007E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A7" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A8" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A9" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" s="3">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A10" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A11" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A12" s="3"/>
+      <c r="B12" s="3"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A13" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="3">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A14" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" s="3">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A15" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B15" s="3">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A16" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16" s="3">
+        <v>0.91</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A17" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17" s="3">
+        <v>0.71</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A19" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="26" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A20" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B20" s="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A21" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B21" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A22" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B22" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A23" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A24" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B24" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A25" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A27" s="16" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A28" s="27" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A29" s="27" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A30" s="27" t="s">
+        <v>94</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3EC3D12-1968-714F-854F-7AA72F889577}">
   <dimension ref="A1:D30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
@@ -30713,7 +30936,7 @@
       <c r="A3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="31">
+      <c r="B3" s="3">
         <v>4</v>
       </c>
     </row>
@@ -30721,7 +30944,7 @@
       <c r="A4" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="32">
+      <c r="B4">
         <v>0.23</v>
       </c>
     </row>
@@ -30729,7 +30952,7 @@
       <c r="A5" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="31">
+      <c r="B5" s="3">
         <v>0.01</v>
       </c>
     </row>
@@ -30737,7 +30960,7 @@
       <c r="A6" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="32">
+      <c r="B6">
         <v>0.01</v>
       </c>
     </row>
@@ -30745,7 +30968,7 @@
       <c r="A7" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="31">
+      <c r="B7" s="3">
         <v>1.2</v>
       </c>
     </row>
@@ -30753,7 +30976,7 @@
       <c r="A8" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="31">
+      <c r="B8" s="3">
         <v>0.5</v>
       </c>
     </row>
@@ -30761,7 +30984,7 @@
       <c r="A9" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="31">
+      <c r="B9" s="3">
         <v>1</v>
       </c>
     </row>
@@ -30769,7 +30992,7 @@
       <c r="A10" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="31">
+      <c r="B10" s="3">
         <v>1</v>
       </c>
     </row>
@@ -30777,7 +31000,7 @@
       <c r="A11" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="31">
+      <c r="B11" s="3">
         <v>1</v>
       </c>
     </row>
@@ -30789,7 +31012,7 @@
       <c r="A13" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="31">
+      <c r="B13" s="3">
         <v>0.2</v>
       </c>
     </row>
@@ -30797,7 +31020,7 @@
       <c r="A14" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="31">
+      <c r="B14" s="3">
         <v>0.6</v>
       </c>
     </row>
@@ -30805,7 +31028,7 @@
       <c r="A15" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="31">
+      <c r="B15" s="3">
         <v>0.3</v>
       </c>
     </row>
@@ -30813,7 +31036,7 @@
       <c r="A16" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="B16" s="31">
+      <c r="B16" s="3">
         <v>0.7</v>
       </c>
     </row>
@@ -30821,7 +31044,7 @@
       <c r="A17" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B17" s="31">
+      <c r="B17" s="3">
         <v>0.5</v>
       </c>
     </row>
@@ -30887,6 +31110,181 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4D0DFFF-026B-7942-BA41-C518504D3FE2}">
+  <dimension ref="A1:B30"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <cols>
+    <col min="1" max="1" width="40.33203125" customWidth="1"/>
+    <col min="2" max="2" width="39.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A1" s="24" t="s">
+        <v>108</v>
+      </c>
+      <c r="B1" s="25"/>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A2" s="3"/>
+      <c r="B2" s="3"/>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="3">
+        <v>2.66</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A4" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A5" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="3"/>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A6" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A7" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="3"/>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A8" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="3"/>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A9" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" s="3"/>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A10" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" s="3"/>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A11" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3"/>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A12" s="3"/>
+      <c r="B12" s="3"/>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A13" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="3"/>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A14" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" s="3"/>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A15" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B15" s="3"/>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A16" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16" s="3"/>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A17" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17" s="3"/>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A19" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="26" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A20" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B20" s="18"/>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A21" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B21" s="3"/>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A22" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B22" s="3"/>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A23" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B23" s="3"/>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A24" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B24" s="3"/>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A25" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B25" s="3"/>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A27" s="16" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A28" s="27" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A29" s="27"/>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A30" s="27"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A28" r:id="rId1" xr:uid="{F07F2465-6662-FA44-B1FA-DB76D168CF25}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{200C08EA-5754-5141-991E-6A7AC4F2528B}">
   <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
@@ -31097,7 +31495,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC1131AB-CE15-5A4C-ABE2-DA91D162E67B}">
   <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
@@ -31301,7 +31699,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62B132E5-5A8B-7C4F-887F-BF1E9B9551E4}">
   <dimension ref="A1:D30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
@@ -31523,7 +31921,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A8F25E9-80DD-4F46-A150-0D1211E7E472}">
   <dimension ref="A1:D30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
@@ -31745,7 +32143,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D68CC4B-0DA8-C14A-B8A7-F18D100FE9A5}">
   <dimension ref="A1:D30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
@@ -31959,7 +32357,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5FD915A-0A31-FD43-A30E-ED6BE6895338}">
   <dimension ref="A1:D30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
@@ -32167,222 +32565,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4966E832-9944-D544-886B-D77EBEEF54A6}">
-  <dimension ref="A1:D30"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
-  <cols>
-    <col min="1" max="1" width="57.5" customWidth="1"/>
-    <col min="2" max="2" width="33" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A1" s="24" t="s">
-        <v>89</v>
-      </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" s="3">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A4" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A5" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B5" s="3">
-        <v>0.14000000000000001</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A6" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6">
-        <v>7.0000000000000007E-2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A7" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7" s="3">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A8" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" s="3">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A9" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B9" s="3">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A10" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B10" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A11" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A13" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B13" s="3">
-        <v>0.3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A14" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B14" s="3">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A15" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B15" s="3">
-        <v>0.3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A16" s="17" t="s">
-        <v>17</v>
-      </c>
-      <c r="B16" s="3">
-        <v>0.91</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A17" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B17" s="3">
-        <v>0.71</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A19" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="B19" s="26" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A20" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B20" s="18">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A21" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B21" s="3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A22" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B22" s="3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A23" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A24" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B24" s="3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A25" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A27" s="16" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A28" s="27" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A29" s="27" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A30" s="27" t="s">
-        <v>94</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>